<commit_message>
Improve grid swapping and adjust cultivation qi costs
</commit_message>
<xml_diff>
--- a/config/xlsx/home_meridians.xlsx
+++ b/config/xlsx/home_meridians.xlsx
@@ -467,12 +467,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>acupoint_rewards</t>
+          <t>acupoint_exp</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>circulation_rewards</t>
+          <t>circulation_exp</t>
         </is>
       </c>
     </row>
@@ -486,17 +486,13 @@
         <v>10</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>42</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -509,17 +505,13 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>57</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -532,17 +524,13 @@
         <v>16</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>72</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -555,17 +543,13 @@
         <v>19</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>87</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -578,17 +562,13 @@
         <v>22</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>102</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="7">
@@ -601,17 +581,13 @@
         <v>25</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>114</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="8">
@@ -624,17 +600,13 @@
         <v>28</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>129</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -647,17 +619,13 @@
         <v>31</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>144</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>121</v>
       </c>
     </row>
     <row r="10">
@@ -670,17 +638,13 @@
         <v>34</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>159</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>160</v>
       </c>
     </row>
     <row r="11">
@@ -693,17 +657,13 @@
         <v>35</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>125</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>375</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -716,17 +676,13 @@
         <v>36</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>130</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>390</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -739,17 +695,13 @@
         <v>37</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>134</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>402</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="14">
@@ -762,17 +714,13 @@
         <v>38</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>139</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>417</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -785,17 +733,13 @@
         <v>39</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>144</v>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>432</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="16">
@@ -808,17 +752,13 @@
         <v>40</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>149</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>447</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="17">
@@ -831,17 +771,13 @@
         <v>41</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>154</v>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>462</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="18">
@@ -854,17 +790,13 @@
         <v>42</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>158</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>474</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="19">
@@ -877,17 +809,13 @@
         <v>43</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>163</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>489</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="20">
@@ -900,17 +828,13 @@
         <v>44</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>168</v>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>504</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="21">
@@ -923,17 +847,13 @@
         <v>35</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>163</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>489</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -946,17 +866,13 @@
         <v>36</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>168</v>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>504</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="23">
@@ -969,17 +885,13 @@
         <v>37</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>173</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>519</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="24">
@@ -992,17 +904,13 @@
         <v>38</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>178</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>534</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="25">
@@ -1015,17 +923,13 @@
         <v>39</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>183</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>549</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="26">
@@ -1038,17 +942,13 @@
         <v>40</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>187</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>561</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -1061,17 +961,13 @@
         <v>41</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>192</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>576</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -1084,17 +980,13 @@
         <v>42</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>197</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>591</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="29">
@@ -1107,17 +999,13 @@
         <v>43</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>202</v>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>606</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="30">
@@ -1130,17 +1018,13 @@
         <v>44</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>207</v>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>621</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="31">
@@ -1153,17 +1037,13 @@
         <v>35</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>211</v>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>633</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="32">
@@ -1176,17 +1056,13 @@
         <v>36</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>216</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>648</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>71</v>
       </c>
     </row>
     <row r="33">
@@ -1199,17 +1075,13 @@
         <v>37</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>221</v>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>663</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="34">
@@ -1222,17 +1094,13 @@
         <v>38</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>226</v>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>678</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>63</v>
       </c>
     </row>
     <row r="35">
@@ -1245,17 +1113,13 @@
         <v>39</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>231</v>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>693</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>59</v>
       </c>
     </row>
     <row r="36">
@@ -1268,17 +1132,13 @@
         <v>40</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>235</v>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>705</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="37">
@@ -1291,17 +1151,13 @@
         <v>41</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>240</v>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>720</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="38">
@@ -1314,17 +1170,13 @@
         <v>42</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>245</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>735</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="39">
@@ -1337,17 +1189,13 @@
         <v>43</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>750</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="40">
@@ -1360,17 +1208,13 @@
         <v>44</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>255</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>765</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="41">
@@ -1383,17 +1227,13 @@
         <v>45</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>269</v>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>807</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="42">
@@ -1406,17 +1246,13 @@
         <v>46</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>274</v>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>822</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>114</v>
       </c>
     </row>
     <row r="43">
@@ -1429,17 +1265,13 @@
         <v>47</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>279</v>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>837</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="44">
@@ -1452,17 +1284,13 @@
         <v>48</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>283</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>849</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="45">
@@ -1475,17 +1303,13 @@
         <v>49</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>288</v>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>864</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="46">
@@ -1498,17 +1322,13 @@
         <v>50</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>293</v>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>879</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="47">
@@ -1521,17 +1341,13 @@
         <v>51</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>298</v>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>894</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>135</v>
       </c>
     </row>
     <row r="48">
@@ -1544,17 +1360,13 @@
         <v>52</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>303</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>909</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="49">
@@ -1567,17 +1379,13 @@
         <v>53</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>307</v>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>921</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="50">
@@ -1590,17 +1398,13 @@
         <v>54</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>312</v>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>936</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="51">
@@ -1613,17 +1417,13 @@
         <v>45</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>346</v>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1038</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="52">
@@ -1636,17 +1436,13 @@
         <v>46</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>351</v>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1053</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="53">
@@ -1659,17 +1455,13 @@
         <v>47</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>355</v>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1065</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="54">
@@ -1682,17 +1474,13 @@
         <v>48</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>360</v>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1080</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="55">
@@ -1705,17 +1493,13 @@
         <v>49</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>365</v>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1095</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>73</v>
       </c>
     </row>
     <row r="56">
@@ -1728,17 +1512,13 @@
         <v>50</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>370</v>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1110</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="57">
@@ -1751,17 +1531,13 @@
         <v>51</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>375</v>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1125</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="58">
@@ -1774,17 +1550,13 @@
         <v>52</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>379</v>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1137</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="59">
@@ -1797,17 +1569,13 @@
         <v>53</v>
       </c>
       <c r="C59" s="3" t="n">
-        <v>384</v>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1152</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="60">
@@ -1820,17 +1588,13 @@
         <v>54</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>389</v>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1167</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="61">
@@ -1843,17 +1607,13 @@
         <v>45</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>442</v>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1326</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>180</v>
       </c>
     </row>
     <row r="62">
@@ -1866,17 +1626,13 @@
         <v>46</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>447</v>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1341</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="63">
@@ -1889,17 +1645,13 @@
         <v>47</v>
       </c>
       <c r="C63" s="3" t="n">
-        <v>451</v>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1353</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>207</v>
       </c>
     </row>
     <row r="64">
@@ -1912,17 +1664,13 @@
         <v>48</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>456</v>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1368</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>198</v>
       </c>
     </row>
     <row r="65">
@@ -1935,17 +1683,13 @@
         <v>49</v>
       </c>
       <c r="C65" s="3" t="n">
-        <v>461</v>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1383</v>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>189</v>
       </c>
     </row>
     <row r="66">
@@ -1958,17 +1702,13 @@
         <v>50</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>466</v>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1398</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>180</v>
       </c>
     </row>
     <row r="67">
@@ -1981,17 +1721,13 @@
         <v>51</v>
       </c>
       <c r="C67" s="3" t="n">
-        <v>471</v>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1413</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>171</v>
       </c>
     </row>
     <row r="68">
@@ -2004,17 +1740,13 @@
         <v>52</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>475</v>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1425</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>214</v>
       </c>
     </row>
     <row r="69">
@@ -2027,17 +1759,13 @@
         <v>53</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>480</v>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1440</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="70">
@@ -2050,17 +1778,13 @@
         <v>54</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>485</v>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1455</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>198</v>
       </c>
     </row>
     <row r="71">
@@ -2073,17 +1797,13 @@
         <v>55</v>
       </c>
       <c r="C71" s="3" t="n">
-        <v>576</v>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1728</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>425</v>
       </c>
     </row>
     <row r="72">
@@ -2096,17 +1816,13 @@
         <v>56</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>581</v>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1743</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>408</v>
       </c>
     </row>
     <row r="73">
@@ -2119,17 +1835,13 @@
         <v>57</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>586</v>
-      </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1758</v>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>391</v>
       </c>
     </row>
     <row r="74">
@@ -2142,17 +1854,13 @@
         <v>58</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>591</v>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1773</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>432</v>
       </c>
     </row>
     <row r="75">
@@ -2165,17 +1873,13 @@
         <v>59</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>596</v>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1788</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>416</v>
       </c>
     </row>
     <row r="76">
@@ -2188,17 +1892,13 @@
         <v>60</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1800</v>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="77">
@@ -2211,17 +1911,13 @@
         <v>61</v>
       </c>
       <c r="C77" s="3" t="n">
-        <v>605</v>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1815</v>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>384</v>
       </c>
     </row>
     <row r="78">
@@ -2234,17 +1930,13 @@
         <v>62</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>610</v>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1830</v>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>430</v>
       </c>
     </row>
     <row r="79">
@@ -2257,17 +1949,13 @@
         <v>63</v>
       </c>
       <c r="C79" s="3" t="n">
-        <v>615</v>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1845</v>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>415</v>
       </c>
     </row>
     <row r="80">
@@ -2280,17 +1968,13 @@
         <v>64</v>
       </c>
       <c r="C80" s="3" t="n">
-        <v>620</v>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>1860</v>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="81">
@@ -2303,17 +1987,13 @@
         <v>55</v>
       </c>
       <c r="C81" s="3" t="n">
-        <v>749</v>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2247</v>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="82">
@@ -2326,17 +2006,13 @@
         <v>56</v>
       </c>
       <c r="C82" s="3" t="n">
-        <v>754</v>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E82" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2262</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>134</v>
       </c>
     </row>
     <row r="83">
@@ -2349,17 +2025,13 @@
         <v>57</v>
       </c>
       <c r="C83" s="3" t="n">
-        <v>759</v>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2277</v>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="84">
@@ -2372,17 +2044,13 @@
         <v>58</v>
       </c>
       <c r="C84" s="3" t="n">
-        <v>764</v>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2292</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>122</v>
       </c>
     </row>
     <row r="85">
@@ -2395,17 +2063,13 @@
         <v>59</v>
       </c>
       <c r="C85" s="3" t="n">
-        <v>768</v>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2304</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="86">
@@ -2418,17 +2082,13 @@
         <v>60</v>
       </c>
       <c r="C86" s="3" t="n">
-        <v>773</v>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E86" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2319</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="87">
@@ -2441,17 +2101,13 @@
         <v>61</v>
       </c>
       <c r="C87" s="3" t="n">
-        <v>778</v>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2334</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>165</v>
       </c>
     </row>
     <row r="88">
@@ -2464,17 +2120,13 @@
         <v>62</v>
       </c>
       <c r="C88" s="3" t="n">
-        <v>783</v>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2349</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>160</v>
       </c>
     </row>
     <row r="89">
@@ -2487,17 +2139,13 @@
         <v>63</v>
       </c>
       <c r="C89" s="3" t="n">
-        <v>788</v>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2364</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>155</v>
       </c>
     </row>
     <row r="90">
@@ -2510,17 +2158,13 @@
         <v>64</v>
       </c>
       <c r="C90" s="3" t="n">
-        <v>792</v>
-      </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E90" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2376</v>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="91">
@@ -2533,17 +2177,13 @@
         <v>55</v>
       </c>
       <c r="C91" s="3" t="n">
-        <v>961</v>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E91" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2883</v>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E91" s="3" t="n">
+        <v>435</v>
       </c>
     </row>
     <row r="92">
@@ -2556,17 +2196,13 @@
         <v>56</v>
       </c>
       <c r="C92" s="3" t="n">
-        <v>965</v>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2895</v>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>418</v>
       </c>
     </row>
     <row r="93">
@@ -2579,17 +2215,13 @@
         <v>57</v>
       </c>
       <c r="C93" s="3" t="n">
-        <v>970</v>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2910</v>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E93" s="3" t="n">
+        <v>401</v>
       </c>
     </row>
     <row r="94">
@@ -2602,17 +2234,13 @@
         <v>58</v>
       </c>
       <c r="C94" s="3" t="n">
-        <v>975</v>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E94" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2925</v>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>384</v>
       </c>
     </row>
     <row r="95">
@@ -2625,17 +2253,13 @@
         <v>59</v>
       </c>
       <c r="C95" s="3" t="n">
-        <v>980</v>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E95" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2940</v>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E95" s="3" t="n">
+        <v>426</v>
       </c>
     </row>
     <row r="96">
@@ -2648,17 +2272,13 @@
         <v>60</v>
       </c>
       <c r="C96" s="3" t="n">
-        <v>985</v>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2955</v>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>410</v>
       </c>
     </row>
     <row r="97">
@@ -2671,17 +2291,13 @@
         <v>61</v>
       </c>
       <c r="C97" s="3" t="n">
-        <v>989</v>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2967</v>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>394</v>
       </c>
     </row>
     <row r="98">
@@ -2694,17 +2310,13 @@
         <v>62</v>
       </c>
       <c r="C98" s="3" t="n">
-        <v>994</v>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2982</v>
+      </c>
+      <c r="D98" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E98" s="3" t="n">
+        <v>440</v>
       </c>
     </row>
     <row r="99">
@@ -2717,17 +2329,13 @@
         <v>63</v>
       </c>
       <c r="C99" s="3" t="n">
-        <v>999</v>
-      </c>
-      <c r="D99" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E99" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>2997</v>
+      </c>
+      <c r="D99" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E99" s="3" t="n">
+        <v>425</v>
       </c>
     </row>
     <row r="100">
@@ -2740,17 +2348,13 @@
         <v>64</v>
       </c>
       <c r="C100" s="3" t="n">
-        <v>1004</v>
-      </c>
-      <c r="D100" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E100" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3012</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>410</v>
       </c>
     </row>
     <row r="101">
@@ -2763,17 +2367,13 @@
         <v>65</v>
       </c>
       <c r="C101" s="3" t="n">
-        <v>1249</v>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3747</v>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>955</v>
       </c>
     </row>
     <row r="102">
@@ -2786,17 +2386,13 @@
         <v>66</v>
       </c>
       <c r="C102" s="3" t="n">
-        <v>1254</v>
-      </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3762</v>
+      </c>
+      <c r="D102" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="E102" s="3" t="n">
+        <v>922</v>
       </c>
     </row>
     <row r="103">
@@ -2809,17 +2405,13 @@
         <v>67</v>
       </c>
       <c r="C103" s="3" t="n">
-        <v>1258</v>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3774</v>
+      </c>
+      <c r="D103" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E103" s="3" t="n">
+        <v>956</v>
       </c>
     </row>
     <row r="104">
@@ -2832,17 +2424,13 @@
         <v>68</v>
       </c>
       <c r="C104" s="3" t="n">
-        <v>1263</v>
-      </c>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3789</v>
+      </c>
+      <c r="D104" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E104" s="3" t="n">
+        <v>924</v>
       </c>
     </row>
     <row r="105">
@@ -2855,17 +2443,13 @@
         <v>69</v>
       </c>
       <c r="C105" s="3" t="n">
-        <v>1268</v>
-      </c>
-      <c r="D105" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E105" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3804</v>
+      </c>
+      <c r="D105" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E105" s="3" t="n">
+        <v>961</v>
       </c>
     </row>
     <row r="106">
@@ -2878,17 +2462,13 @@
         <v>70</v>
       </c>
       <c r="C106" s="3" t="n">
-        <v>1273</v>
-      </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E106" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3819</v>
+      </c>
+      <c r="D106" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E106" s="3" t="n">
+        <v>930</v>
       </c>
     </row>
     <row r="107">
@@ -2901,17 +2481,13 @@
         <v>71</v>
       </c>
       <c r="C107" s="3" t="n">
-        <v>1278</v>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3834</v>
+      </c>
+      <c r="D107" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E107" s="3" t="n">
+        <v>899</v>
       </c>
     </row>
     <row r="108">
@@ -2924,17 +2500,13 @@
         <v>72</v>
       </c>
       <c r="C108" s="3" t="n">
-        <v>1282</v>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3846</v>
+      </c>
+      <c r="D108" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E108" s="3" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="109">
@@ -2947,17 +2519,13 @@
         <v>73</v>
       </c>
       <c r="C109" s="3" t="n">
-        <v>1287</v>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3861</v>
+      </c>
+      <c r="D109" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>910</v>
       </c>
     </row>
     <row r="110">
@@ -2970,17 +2538,13 @@
         <v>74</v>
       </c>
       <c r="C110" s="3" t="n">
-        <v>1292</v>
-      </c>
-      <c r="D110" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:15</t>
-        </is>
-      </c>
-      <c r="E110" s="3" t="inlineStr">
-        <is>
-          <t>4:0;3:100</t>
-        </is>
+        <v>3876</v>
+      </c>
+      <c r="D110" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="E110" s="3" t="n">
+        <v>954</v>
       </c>
     </row>
   </sheetData>

</xml_diff>